<commit_message>
Actualizar datos de Grupos_66 y eliminar Grupos_66-Quito
</commit_message>
<xml_diff>
--- a/src/assets/data/Grupos_66.xlsx
+++ b/src/assets/data/Grupos_66.xlsx
@@ -496,13 +496,13 @@
         <x:v>0909119299</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -592,7 +592,7 @@
         <x:v>Grupo 4 - Aula D203</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -621,13 +621,13 @@
         <x:v>Grupo 5 - Aula D204</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="65" customHeight="1">
@@ -757,13 +757,13 @@
         <x:v>0922639752</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -824,13 +824,13 @@
         <x:v>Grupo 3 - Aula D202</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H13" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="65" customHeight="1">
@@ -998,13 +998,13 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G19" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H19" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="65" customHeight="1">
@@ -1018,13 +1018,13 @@
         <x:v>0102054871</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G20" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -1172,13 +1172,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G25" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H25" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I25" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="65" customHeight="1">
@@ -1279,13 +1279,13 @@
         <x:v>0910743954</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -1404,13 +1404,13 @@
         <x:v>Grupo 5 - Aula D204</x:v>
       </x:c>
       <x:c r="G33" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H33" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I33" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="65" customHeight="1">
@@ -1491,7 +1491,7 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G36" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H36" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -1540,13 +1540,13 @@
         <x:v>0914078290</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E38" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F38" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G38" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -1636,7 +1636,7 @@
         <x:v>Grupo 4 - Aula D203</x:v>
       </x:c>
       <x:c r="G41" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H41" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -1801,13 +1801,13 @@
         <x:v>0202336749</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F47" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G47" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -2013,13 +2013,13 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G54" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H54" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I54" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="65" customHeight="1">
@@ -2062,13 +2062,13 @@
         <x:v>1102293402</x:v>
       </x:c>
       <x:c r="D56" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F56" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G56" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -2323,13 +2323,13 @@
         <x:v>1204922544</x:v>
       </x:c>
       <x:c r="D65" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E65" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F65" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G65" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -2361,13 +2361,13 @@
         <x:v>Grupo 2 - Aula D201</x:v>
       </x:c>
       <x:c r="G66" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H66" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I66" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="65" customHeight="1">
@@ -2584,13 +2584,13 @@
         <x:v>0919123067</x:v>
       </x:c>
       <x:c r="D74" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E74" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F74" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G74" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -2738,13 +2738,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G79" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H79" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I79" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="65" customHeight="1">
@@ -2767,7 +2767,7 @@
         <x:v>Grupo 7 - Aula D206</x:v>
       </x:c>
       <x:c r="G80" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H80" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -2845,22 +2845,22 @@
         <x:v>0916168784</x:v>
       </x:c>
       <x:c r="D83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I83" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="65" customHeight="1">
@@ -2912,13 +2912,13 @@
         <x:v>Grupo 3 - Aula D202</x:v>
       </x:c>
       <x:c r="G85" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H85" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I85" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="65" customHeight="1">
@@ -3057,7 +3057,7 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G90" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H90" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -3106,13 +3106,13 @@
         <x:v>0921267951</x:v>
       </x:c>
       <x:c r="D92" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E92" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F92" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G92" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -3318,13 +3318,13 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G99" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H99" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I99" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="65" customHeight="1">
@@ -3367,13 +3367,13 @@
         <x:v>0914335484</x:v>
       </x:c>
       <x:c r="D101" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E101" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F101" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G101" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -3405,13 +3405,13 @@
         <x:v>Grupo 2 - Aula D201</x:v>
       </x:c>
       <x:c r="G102" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H102" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I102" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="65" customHeight="1">
@@ -3550,13 +3550,13 @@
         <x:v>Grupo 7 - Aula D206</x:v>
       </x:c>
       <x:c r="G107" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H107" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I107" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="65" customHeight="1">
@@ -3608,13 +3608,13 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G109" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H109" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I109" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="65" customHeight="1">
@@ -3628,13 +3628,13 @@
         <x:v>0917208084</x:v>
       </x:c>
       <x:c r="D110" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E110" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F110" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G110" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -3889,13 +3889,13 @@
         <x:v>0911019529</x:v>
       </x:c>
       <x:c r="D119" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E119" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F119" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G119" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -4043,7 +4043,7 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G124" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H124" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -4130,13 +4130,13 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G127" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H127" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I127" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="65" customHeight="1">
@@ -4150,13 +4150,13 @@
         <x:v>0915336945</x:v>
       </x:c>
       <x:c r="D128" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E128" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F128" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G128" s="9" t="str">
         <x:v>Grupo 8 - Aula por confirmar</x:v>
@@ -4333,13 +4333,13 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G134" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H134" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I134" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="65" customHeight="1">
@@ -4382,13 +4382,13 @@
         <x:v>0926684325</x:v>
       </x:c>
       <x:c r="D136" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E136" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F136" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G136" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -4420,13 +4420,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G137" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H137" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I137" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="65" customHeight="1">
@@ -4507,13 +4507,13 @@
         <x:v>Grupo 4 - Aula D203</x:v>
       </x:c>
       <x:c r="G140" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H140" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I140" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="65" customHeight="1">
@@ -4652,7 +4652,7 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G145" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H145" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -4672,13 +4672,13 @@
         <x:v>0930340112</x:v>
       </x:c>
       <x:c r="D146" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E146" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F146" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G146" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -4768,13 +4768,13 @@
         <x:v>Grupo 4 - Aula D203</x:v>
       </x:c>
       <x:c r="G149" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H149" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I149" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="65" customHeight="1">
@@ -4933,13 +4933,13 @@
         <x:v>0919514117</x:v>
       </x:c>
       <x:c r="D155" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E155" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F155" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G155" s="9" t="str">
         <x:v>Grupo 7 - Aula D206</x:v>
@@ -4971,7 +4971,7 @@
         <x:v>Grupo 2 - Aula D201</x:v>
       </x:c>
       <x:c r="G156" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H156" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -5000,13 +5000,13 @@
         <x:v>Grupo 3 - Aula D202</x:v>
       </x:c>
       <x:c r="G157" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H157" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I157" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="65" customHeight="1">
@@ -5116,13 +5116,13 @@
         <x:v>Grupo 7 - Aula D206</x:v>
       </x:c>
       <x:c r="G161" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H161" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I161" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="65" customHeight="1">
@@ -5194,13 +5194,13 @@
         <x:v>0914286042</x:v>
       </x:c>
       <x:c r="D164" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E164" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F164" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G164" s="9" t="str">
         <x:v>Grupo 8 - Aula por confirmar</x:v>
@@ -5319,7 +5319,7 @@
         <x:v>Grupo 5 - Aula D204</x:v>
       </x:c>
       <x:c r="G168" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H168" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -5348,7 +5348,7 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G169" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H169" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -5455,13 +5455,13 @@
         <x:v>0905056016</x:v>
       </x:c>
       <x:c r="D173" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E173" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F173" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G173" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -5696,13 +5696,13 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G181" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H181" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I181" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="65" customHeight="1">
@@ -5716,13 +5716,13 @@
         <x:v>1310835457</x:v>
       </x:c>
       <x:c r="D182" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E182" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F182" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G182" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -5977,13 +5977,13 @@
         <x:v>1755500665</x:v>
       </x:c>
       <x:c r="D191" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E191" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F191" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G191" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -6218,7 +6218,7 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G199" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H199" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -6238,13 +6238,13 @@
         <x:v>0602579948</x:v>
       </x:c>
       <x:c r="D200" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E200" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F200" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G200" s="9" t="str">
         <x:v>Grupo 3 - Aula D202</x:v>
@@ -6499,13 +6499,13 @@
         <x:v>0912155652</x:v>
       </x:c>
       <x:c r="D209" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E209" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F209" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G209" s="9" t="str">
         <x:v>Grupo 6 - Aula D205</x:v>
@@ -6566,13 +6566,13 @@
         <x:v>Grupo 3 - Aula D202</x:v>
       </x:c>
       <x:c r="G211" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H211" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I211" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="65" customHeight="1">
@@ -6653,7 +6653,7 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G214" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H214" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -6760,13 +6760,13 @@
         <x:v>0922799655</x:v>
       </x:c>
       <x:c r="D218" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E218" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F218" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G218" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -7021,13 +7021,13 @@
         <x:v>0917494890</x:v>
       </x:c>
       <x:c r="D227" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E227" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F227" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G227" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -7282,13 +7282,13 @@
         <x:v>0602162539</x:v>
       </x:c>
       <x:c r="D236" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E236" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F236" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G236" s="9" t="str">
         <x:v>Grupo 6 - Aula D205</x:v>
@@ -7349,7 +7349,7 @@
         <x:v>Grupo 3 - Aula D202</x:v>
       </x:c>
       <x:c r="G238" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H238" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -7436,13 +7436,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G241" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H241" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I241" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="65" customHeight="1">
@@ -7543,16 +7543,16 @@
         <x:v>0910952571</x:v>
       </x:c>
       <x:c r="D245" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E245" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F245" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G245" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H245" s="9" t="str">
         <x:v>No Convocado</x:v>
@@ -7804,13 +7804,13 @@
         <x:v>0924194889</x:v>
       </x:c>
       <x:c r="D254" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E254" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F254" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G254" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -7958,13 +7958,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G259" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H259" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I259" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="260" ht="65" customHeight="1">
@@ -8065,13 +8065,13 @@
         <x:v>0917242448</x:v>
       </x:c>
       <x:c r="D263" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E263" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F263" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G263" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -8324,13 +8324,13 @@
         <x:v>0950594754</x:v>
       </x:c>
       <x:c r="D272" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E272" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F272" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G272" s="9" t="str">
         <x:v>Grupo 5 - Aula D204</x:v>
@@ -8585,13 +8585,13 @@
         <x:v>1705290128</x:v>
       </x:c>
       <x:c r="D281" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E281" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F281" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G281" s="9" t="str">
         <x:v>Grupo 4 - Aula D203</x:v>
@@ -8623,13 +8623,13 @@
         <x:v>Grupo 2 - Aula D201</x:v>
       </x:c>
       <x:c r="G282" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H282" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I282" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="283" ht="65" customHeight="1">
@@ -8797,13 +8797,13 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G288" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H288" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I288" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="289" ht="65" customHeight="1">
@@ -8817,22 +8817,22 @@
         <x:v>1204142937</x:v>
       </x:c>
       <x:c r="D289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I289" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="290" ht="65" customHeight="1">
@@ -9000,13 +9000,13 @@
         <x:v>Grupo 6 - Aula D205</x:v>
       </x:c>
       <x:c r="G295" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H295" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I295" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="296" ht="65" customHeight="1">
@@ -9058,13 +9058,13 @@
         <x:v>Grupo 8 - Aula D207</x:v>
       </x:c>
       <x:c r="G297" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H297" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I297" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="298" ht="65" customHeight="1">
@@ -9087,13 +9087,13 @@
         <x:v>Grupo 9 - Aula D208</x:v>
       </x:c>
       <x:c r="G298" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H298" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I298" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
     <x:row r="299" ht="65" customHeight="1">
@@ -9107,22 +9107,22 @@
         <x:v>0917375537</x:v>
       </x:c>
       <x:c r="D299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="H299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="I299" s="9" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10626,7 +10626,7 @@
     </x:row>
     <x:row r="3" ht="93" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
         <x:v>FABIÁN LEONARDO CUESTA ASTUDILLO (DIRECTOR NACIONAL)
@@ -10884,7 +10884,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -10914,7 +10914,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D4" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -10944,7 +10944,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -10974,7 +10974,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11004,7 +11004,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11034,7 +11034,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11064,7 +11064,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11094,7 +11094,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11124,7 +11124,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11154,7 +11154,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11184,7 +11184,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
         <x:v>MAESTRIA EN GERENCIA TRIBUTARIA</x:v>
@@ -11214,7 +11214,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11244,7 +11244,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
         <x:v>DIRECCION TECNICA DE PLANEACION EVALUACION Y ACREDITACION</x:v>
@@ -11274,7 +11274,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -11304,7 +11304,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11334,7 +11334,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D18" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11364,7 +11364,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11394,7 +11394,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D20" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11424,7 +11424,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D21" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11454,7 +11454,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -11484,7 +11484,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D23" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11514,7 +11514,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -11544,7 +11544,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -11574,7 +11574,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D26" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11604,7 +11604,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D27" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -11634,7 +11634,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -11664,7 +11664,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11694,7 +11694,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D30" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -11724,7 +11724,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -11754,7 +11754,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11784,7 +11784,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -11814,7 +11814,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -16275,7 +16275,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
@@ -16297,8 +16297,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
         <x:v>lalarcon@ups.edu.ec</x:v>
@@ -16451,8 +16451,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
         <x:v>eandradee@ups.edu.ec</x:v>
@@ -16583,8 +16583,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
         <x:v>kascencio@ups.edu.ec</x:v>
@@ -16715,8 +16715,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
         <x:v>jbalas@ups.edu.ec</x:v>
@@ -16891,8 +16891,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
         <x:v>mbastidas@ups.edu.ec</x:v>
@@ -16957,7 +16957,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
@@ -17067,7 +17067,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D41" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
@@ -17353,8 +17353,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D54" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E54" s="4" t="str">
         <x:v>jcarreraj@ups.edu.ec</x:v>
@@ -17617,8 +17617,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D66" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E66" s="4" t="str">
         <x:v>mchavez@ups.edu.ec</x:v>
@@ -17903,8 +17903,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D79" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E79" s="4" t="str">
         <x:v>jcueva@ups.edu.ec</x:v>
@@ -17925,7 +17925,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D80" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E80" s="4" t="str">
@@ -17991,8 +17991,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D83" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E83" s="4" t="str">
         <x:v>ddefas@ups.edu.ec</x:v>
@@ -18035,8 +18035,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D85" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E85" s="4" t="str">
         <x:v>sdelgadof@ups.edu.ec</x:v>
@@ -18145,7 +18145,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D90" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E90" s="4" t="str">
@@ -18343,8 +18343,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D99" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E99" s="4" t="str">
         <x:v>gespinozar@ups.edu.ec</x:v>
@@ -18409,8 +18409,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D102" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E102" s="4" t="str">
         <x:v>ofiallos@ups.edu.ec</x:v>
@@ -18519,8 +18519,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D107" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E107" s="4" t="str">
         <x:v>efranco@ups.edu.ec</x:v>
@@ -18563,8 +18563,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D109" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E109" s="4" t="str">
         <x:v>jfreirem@ups.edu.ec</x:v>
@@ -18893,7 +18893,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D124" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E124" s="4" t="str">
@@ -18959,8 +18959,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D127" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E127" s="4" t="str">
         <x:v>fherrera@ups.edu.ec</x:v>
@@ -19113,8 +19113,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D134" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E134" s="4" t="str">
         <x:v>eissa@ups.edu.ec</x:v>
@@ -19179,8 +19179,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D137" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E137" s="4" t="str">
         <x:v>hiniguez@ups.edu.ec</x:v>
@@ -19245,8 +19245,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D140" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E140" s="4" t="str">
         <x:v>mjaram@ups.edu.ec</x:v>
@@ -19355,7 +19355,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D145" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E145" s="4" t="str">
@@ -19443,8 +19443,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D149" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E149" s="4" t="str">
         <x:v>fleonb@ups.edu.ec</x:v>
@@ -19597,7 +19597,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D156" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E156" s="4" t="str">
@@ -19619,8 +19619,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D157" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E157" s="4" t="str">
         <x:v>alopezn@ups.edu.ec</x:v>
@@ -19707,8 +19707,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D161" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E161" s="4" t="str">
         <x:v>alozano@ups.edu.ec</x:v>
@@ -19861,7 +19861,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D168" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E168" s="4" t="str">
@@ -19883,7 +19883,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D169" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E169" s="4" t="str">
@@ -20147,8 +20147,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D181" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E181" s="4" t="str">
         <x:v>jmorenod@ups.edu.ec</x:v>
@@ -20543,7 +20543,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D199" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E199" s="4" t="str">
@@ -20807,8 +20807,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D211" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E211" s="4" t="str">
         <x:v>spozo@ups.edu.ec</x:v>
@@ -20873,7 +20873,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D214" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E214" s="4" t="str">
@@ -21401,7 +21401,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D238" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E238" s="4" t="str">
@@ -21467,8 +21467,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D241" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E241" s="4" t="str">
         <x:v>esalazar@ups.edu.ec</x:v>
@@ -21555,7 +21555,7 @@
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="D245" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
+        <x:v>T4: Grupo 1 - Aula D209
 T5 y T6: No Convocado</x:v>
       </x:c>
       <x:c r="E245" s="4" t="str">
@@ -21863,8 +21863,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D259" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E259" s="4" t="str">
         <x:v>nsumba@ups.edu.ec</x:v>
@@ -22367,8 +22367,8 @@
 T5 y T6: DIRECTOR/A DE CARRERA (convocado por responsabilidad de carrera)</x:v>
       </x:c>
       <x:c r="D282" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E282" s="4" t="str">
         <x:v>kvallejo@ups.edu.ec</x:v>
@@ -22499,8 +22499,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D288" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E288" s="4" t="str">
         <x:v>vvera@ups.edu.ec</x:v>
@@ -22521,8 +22521,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D289" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E289" s="4" t="str">
         <x:v>fvillacres@ups.edu.ec</x:v>
@@ -22653,8 +22653,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D295" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E295" s="4" t="str">
         <x:v>tyaguana@ups.edu.ec</x:v>
@@ -22697,8 +22697,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D297" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E297" s="4" t="str">
         <x:v>fzambrano@ups.edu.ec</x:v>
@@ -22719,8 +22719,8 @@
 T5 y T6: PARTICIPANTE</x:v>
       </x:c>
       <x:c r="D298" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E298" s="4" t="str">
         <x:v>nzea@ups.edu.ec</x:v>
@@ -22741,8 +22741,8 @@
 T5 y T6: RESP. AREA CONOC. SEDE</x:v>
       </x:c>
       <x:c r="D299" s="4" t="str">
-        <x:v>T4: Grupo 1 - Aula D200
-T5 y T6: Grupo 1 - Aula D200</x:v>
+        <x:v>T4: Grupo 1 - Aula D209
+T5 y T6: Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="E299" s="4" t="str">
         <x:v>mzunigaa@ups.edu.ec</x:v>
@@ -23272,7 +23272,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="11" t="str">
-        <x:v>TALLERES 1, 2 Y 3 — Lunes 12 y martes 13 de octubre — Grupo 1 — Campus Centenario - Edif. D - Piso 1 - Aula D200</x:v>
+        <x:v>TALLERES 1, 2 Y 3 — Lunes 12 y martes 13 de octubre — Grupo 1 — Campus Centenario - Edif. D - Piso 1 - Aula D209</x:v>
       </x:c>
       <x:c r="B1" s="11"/>
       <x:c r="C1" s="11"/>
@@ -23323,7 +23323,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
         <x:v>INGENIERIA AUTOMOTRIZ</x:v>
@@ -23352,7 +23352,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D4" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
         <x:v>ELECTRONICA Y AUTOMATIZACION</x:v>
@@ -23381,7 +23381,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
         <x:v>INGENIERIA ELECTRICA</x:v>
@@ -23410,7 +23410,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
         <x:v>ODONTOLOGIA</x:v>
@@ -23439,7 +23439,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
         <x:v>INGENIERIA AMBIENTAL</x:v>
@@ -23468,7 +23468,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
         <x:v>INGENIERIA AUTOMOTRIZ</x:v>
@@ -23497,7 +23497,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
         <x:v>TELECOMUNICACIONES</x:v>
@@ -23526,7 +23526,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
         <x:v>INGENIERIA CIVIL</x:v>
@@ -23555,7 +23555,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
         <x:v>TELECOMUNICACIONES</x:v>
@@ -23584,7 +23584,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -23613,7 +23613,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
         <x:v>PSICOLOGIA CLINICA</x:v>
@@ -23642,7 +23642,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
         <x:v>MECATRONICA</x:v>
@@ -23671,7 +23671,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
         <x:v>ELECTRONICA Y AUTOMATIZACION</x:v>
@@ -23700,7 +23700,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
         <x:v>INGENIERIA INDUSTRIAL</x:v>
@@ -23729,7 +23729,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
         <x:v>INSTITUTO DE IDIOMAS</x:v>
@@ -23758,7 +23758,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D18" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
         <x:v>ODONTOLOGIA</x:v>
@@ -23787,7 +23787,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
         <x:v>ODONTOLOGIA</x:v>
@@ -23816,7 +23816,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D20" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
         <x:v>TEOLOGIA MODALIDAD EN LINEA</x:v>
@@ -23845,7 +23845,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D21" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
         <x:v>INSTITUTO DE IDIOMAS</x:v>
@@ -23874,7 +23874,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
         <x:v>INGENIERIA INDUSTRIAL</x:v>
@@ -23903,7 +23903,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D23" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
         <x:v>INGENIERIA CIVIL</x:v>
@@ -23932,7 +23932,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
         <x:v>ODONTOLOGIA</x:v>
@@ -23961,7 +23961,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
         <x:v>COORDINACIÓN DE DESARROLLO ACADÉMICO</x:v>
@@ -23990,7 +23990,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D26" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
         <x:v>EDUCACION INICIAL</x:v>
@@ -24019,7 +24019,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D27" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
         <x:v>MAESTRIA EN ANALITICA DE DATOS</x:v>
@@ -24048,7 +24048,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
         <x:v>ODONTOLOGIA</x:v>
@@ -24077,7 +24077,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
         <x:v>PEDAGOGIA DE LA ACTIVIDAD FISICA</x:v>
@@ -24106,7 +24106,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D30" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -24135,7 +24135,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
         <x:v>PSICOLOGIA CLINICA</x:v>
@@ -24164,7 +24164,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
         <x:v>INGENIERIA INDUSTRIAL</x:v>
@@ -24193,7 +24193,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
         <x:v>PSICOLOGIA CLINICA</x:v>
@@ -24222,7 +24222,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
         <x:v>ARQUITECTURA</x:v>
@@ -24251,7 +24251,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D35" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E35" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -24280,7 +24280,7 @@
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -31517,7 +31517,7 @@
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
         <x:v>FLORALBA DEL ROCIO AGUILAR GORDON</x:v>
@@ -31695,7 +31695,7 @@
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
       <x:c r="A16" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="B16" s="4" t="str">
         <x:v>Administración y economía</x:v>
@@ -32905,7 +32905,7 @@
         <x:v>Grupo 1</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="C3" s="14" t="n">
         <x:f>'T5-6 Resumen'!D3</x:f>
@@ -33725,10 +33725,10 @@
         <x:v>0916656408</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G12" s="4" t="str">
         <x:v>SI</x:v>
@@ -34011,10 +34011,10 @@
         <x:v>0917770778</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F23" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G23" s="4" t="str">
         <x:v>NO</x:v>
@@ -34037,10 +34037,10 @@
         <x:v>1204142937</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G24" s="4" t="str">
         <x:v>SI</x:v>
@@ -34089,10 +34089,10 @@
         <x:v>0917360554</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
-        <x:v>Grupo 1 - Aula D200</x:v>
+        <x:v>Grupo 1 - Aula D209</x:v>
       </x:c>
       <x:c r="G26" s="4" t="str">
         <x:v>SI</x:v>
@@ -34164,7 +34164,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
         <x:v>FABIÁN LEONARDO CUESTA ASTUDILLO (DIRECTOR NACIONAL)
@@ -34413,7 +34413,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34443,7 +34443,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D4" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -34473,7 +34473,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -34503,7 +34503,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34533,7 +34533,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34563,7 +34563,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34593,7 +34593,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -34623,7 +34623,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -34653,7 +34653,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34683,7 +34683,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -34713,7 +34713,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34743,7 +34743,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34773,7 +34773,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -34803,7 +34803,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34833,7 +34833,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34863,7 +34863,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D18" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
         <x:v>MAESTRIA EN GERENCIA TRIBUTARIA</x:v>
@@ -34893,7 +34893,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -34923,7 +34923,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D20" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
         <x:v>DIRECCION TECNICA DE PLANEACION EVALUACION Y ACREDITACION</x:v>
@@ -34953,7 +34953,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D21" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -34983,7 +34983,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35013,7 +35013,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D23" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35043,7 +35043,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35073,7 +35073,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35103,7 +35103,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D26" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35133,7 +35133,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D27" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
         <x:v>VICERRECTORADO DE SEDE</x:v>
@@ -35163,7 +35163,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35193,7 +35193,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35223,7 +35223,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D30" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -35253,7 +35253,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35283,7 +35283,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
         <x:v>DIRECCION TECNICA DE VINCULACION CON LA SOCIEDAD</x:v>
@@ -35313,7 +35313,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35343,7 +35343,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -35373,7 +35373,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D35" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E35" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35403,7 +35403,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -35433,7 +35433,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D37" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E37" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35463,7 +35463,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D38" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E38" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35493,7 +35493,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D39" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E39" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35523,7 +35523,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35553,7 +35553,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D41" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
         <x:v>ADMINISTRACION DE EMPRESAS</x:v>
@@ -35583,7 +35583,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D42" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
         <x:v>ECONOMIA</x:v>
@@ -35613,7 +35613,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D43" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E43" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35643,7 +35643,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D44" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E44" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -35673,7 +35673,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D45" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E45" s="4" t="str">
         <x:v>NEGOCIOS DIGITALES</x:v>
@@ -35703,7 +35703,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D46" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E46" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35733,7 +35733,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D47" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E47" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>
@@ -35763,7 +35763,7 @@
 ZUÑIGA ALVARADO MARIA ALEJANDRA (RESPONSABLE SEDE)</x:v>
       </x:c>
       <x:c r="D48" s="4" t="str">
-        <x:v>Aula D200</x:v>
+        <x:v>Aula D209</x:v>
       </x:c>
       <x:c r="E48" s="4" t="str">
         <x:v>CONTABILIDAD Y AUDITORIA</x:v>

</xml_diff>